<commit_message>
Update regression scripts to reflect new training, validation, and test year ranges. Refactor data processing to dynamically generate file names and labels based on updated periods. Enhance lagged column handling in fixed effects model to ensure proper data integrity and prevent empty validation/test splits.
</commit_message>
<xml_diff>
--- a/Good one/3. Regression/3.1_split_data/Imbalance_table.xlsx
+++ b/Good one/3. Regression/3.1_split_data/Imbalance_table.xlsx
@@ -453,50 +453,48 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Train (1985-2007)</t>
+          <t>Train (1985-2016)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5175</v>
+        <v>7200</v>
       </c>
       <c r="C2" t="n">
-        <v>302</v>
+        <v>405</v>
       </c>
       <c r="D2" t="n">
-        <v>6.14</v>
+        <v>5.91</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Validation (2008-2010)</t>
+          <t>Validation (2017-2019)</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>675</v>
       </c>
       <c r="C3" t="n">
-        <v>63</v>
+        <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>9.81</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Test (2011-2021)</t>
+          <t>Test (2020-2021)</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2475</v>
+        <v>450</v>
       </c>
       <c r="C4" t="n">
-        <v>43</v>
-      </c>
-      <c r="D4" t="n">
-        <v>2.87</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update training, validation, and test year ranges in regression scripts. Refactor file path generation for datasets and adjust output labels accordingly. Remove outdated Excel file to streamline project structure.
</commit_message>
<xml_diff>
--- a/Good one/3. Regression/3.1_split_data/Imbalance_table.xlsx
+++ b/Good one/3. Regression/3.1_split_data/Imbalance_table.xlsx
@@ -453,48 +453,50 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Train (1985-2016)</t>
+          <t>Train (1985-2013)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7200</v>
+        <v>6525</v>
       </c>
       <c r="C2" t="n">
-        <v>405</v>
+        <v>394</v>
       </c>
       <c r="D2" t="n">
-        <v>5.91</v>
+        <v>6.35</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Validation (2017-2019)</t>
+          <t>Validation (2014-2015)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>675</v>
+        <v>450</v>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D3" t="n">
-        <v>1.4</v>
+        <v>1.87</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Test (2020-2021)</t>
+          <t>Test (2016-2017)</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>450</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" t="inlineStr"/>
+        <v>6</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.4</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>